<commit_message>
feat(seo): add verified answer intent coverage
Add a dedicated FAQ page, local map and delivery coverage, internal links from intent pages, and a transparent disposition for all 500 researched keywords.

Co-authored-by: hmad28 <email1.hammad@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/LalaGiDimsum_Keyword_Map.xlsx
+++ b/docs/LalaGiDimsum_Keyword_Map.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementasi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="500 Keywords" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Kategori" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kebijakan Keyword" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="500 Keywords" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Kategori" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Implementasi'!$A$1:$D$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'500 Keywords'!$A$1:$J$501</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'500 Keywords'!$A$1:$J$501</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -552,7 +553,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Tabel harga aktual + FAQ + Product/Offer</t>
+          <t>Katalog approved tetap utuh + metadata + Product/Offer nonvisual</t>
         </is>
       </c>
     </row>
@@ -619,6 +620,28 @@
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Fakta brand + nomor halal + jam layanan + kanal resmi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>/faq</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>AEO: harga, menu, halal, pemesanan, dan pengiriman</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>FAQ LalaGi Dimsum | Harga, Pemesanan &amp; Pengiriman</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Jawaban langsung berbasis fakta + FAQPage + Breadcrumb</t>
         </is>
       </c>
     </row>
@@ -629,6 +652,110 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Arti</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Tindakan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Diimplementasikan</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Intent valid dan didukung fakta bisnis</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Ditargetkan lewat halaman, metadata, copy, FAQ, atau structured data yang relevan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Variasi semantik</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Variasi query lokasi atau modifier subjektif</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Dipakai untuk riset/discovery tanpa klaim berlebihan dan tanpa doorway page</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Butuh verifikasi</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Memerlukan SOP resmi dari client</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Tidak dipublikasikan sampai ada jawaban operasional yang disetujui</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Ditahan</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Produk, kanal, atau layanan belum tersedia/terverifikasi</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Tidak ditargetkan agar website tidak membuat klaim palsu</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1693,7 +1820,7 @@
       </c>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2566,7 @@
       </c>
       <c r="J36" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -3134,12 +3261,12 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J50" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3184,12 +3311,12 @@
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J51" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3234,12 +3361,12 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J52" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3284,12 +3411,12 @@
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J53" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3334,12 +3461,12 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J54" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3384,12 +3511,12 @@
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J55" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3434,12 +3561,12 @@
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J56" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3484,12 +3611,12 @@
       </c>
       <c r="I57" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J57" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3534,12 +3661,12 @@
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J58" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3711,12 @@
       </c>
       <c r="I59" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J59" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3634,12 +3761,12 @@
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J60" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3684,12 +3811,12 @@
       </c>
       <c r="I61" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J61" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3734,12 +3861,12 @@
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J62" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3784,12 +3911,12 @@
       </c>
       <c r="I63" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J63" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3834,12 +3961,12 @@
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J64" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3884,12 +4011,12 @@
       </c>
       <c r="I65" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J65" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3934,12 +4061,12 @@
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J66" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -3984,12 +4111,12 @@
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J67" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4034,12 +4161,12 @@
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J68" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4084,12 +4211,12 @@
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J69" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4134,12 +4261,12 @@
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J70" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4184,12 +4311,12 @@
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J71" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4384,12 +4511,12 @@
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J75" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4434,12 +4561,12 @@
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J76" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4484,12 +4611,12 @@
       </c>
       <c r="I77" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J77" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4534,12 +4661,12 @@
       </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J78" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4584,12 +4711,12 @@
       </c>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J79" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4634,12 +4761,12 @@
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J80" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4684,12 +4811,12 @@
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J81" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4734,12 +4861,12 @@
       </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J82" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4784,12 +4911,12 @@
       </c>
       <c r="I83" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J83" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4834,12 +4961,12 @@
       </c>
       <c r="I84" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J84" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4884,12 +5011,12 @@
       </c>
       <c r="I85" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J85" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4934,12 +5061,12 @@
       </c>
       <c r="I86" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J86" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -4984,12 +5111,12 @@
       </c>
       <c r="I87" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J87" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5034,12 +5161,12 @@
       </c>
       <c r="I88" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J88" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5084,12 +5211,12 @@
       </c>
       <c r="I89" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J89" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5134,12 +5261,12 @@
       </c>
       <c r="I90" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J90" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5184,12 +5311,12 @@
       </c>
       <c r="I91" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J91" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5234,12 +5361,12 @@
       </c>
       <c r="I92" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J92" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5284,12 +5411,12 @@
       </c>
       <c r="I93" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J93" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5334,12 +5461,12 @@
       </c>
       <c r="I94" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J94" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5384,12 +5511,12 @@
       </c>
       <c r="I95" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J95" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5434,12 +5561,12 @@
       </c>
       <c r="I96" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J96" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5634,12 +5761,12 @@
       </c>
       <c r="I100" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J100" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5684,12 +5811,12 @@
       </c>
       <c r="I101" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J101" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5734,12 +5861,12 @@
       </c>
       <c r="I102" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J102" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5784,12 +5911,12 @@
       </c>
       <c r="I103" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J103" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5834,12 +5961,12 @@
       </c>
       <c r="I104" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J104" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5884,12 +6011,12 @@
       </c>
       <c r="I105" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J105" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5934,12 +6061,12 @@
       </c>
       <c r="I106" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J106" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -5984,12 +6111,12 @@
       </c>
       <c r="I107" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J107" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6034,12 +6161,12 @@
       </c>
       <c r="I108" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J108" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6084,12 +6211,12 @@
       </c>
       <c r="I109" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J109" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6134,12 +6261,12 @@
       </c>
       <c r="I110" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J110" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6184,12 +6311,12 @@
       </c>
       <c r="I111" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J111" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6234,12 +6361,12 @@
       </c>
       <c r="I112" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J112" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6284,12 +6411,12 @@
       </c>
       <c r="I113" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J113" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6334,12 +6461,12 @@
       </c>
       <c r="I114" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J114" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6384,12 +6511,12 @@
       </c>
       <c r="I115" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J115" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6434,12 +6561,12 @@
       </c>
       <c r="I116" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J116" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6484,12 +6611,12 @@
       </c>
       <c r="I117" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J117" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6534,12 +6661,12 @@
       </c>
       <c r="I118" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J118" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6584,12 +6711,12 @@
       </c>
       <c r="I119" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J119" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6634,12 +6761,12 @@
       </c>
       <c r="I120" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J120" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6684,12 +6811,12 @@
       </c>
       <c r="I121" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J121" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6884,12 +7011,12 @@
       </c>
       <c r="I125" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J125" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6934,12 +7061,12 @@
       </c>
       <c r="I126" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J126" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -6984,12 +7111,12 @@
       </c>
       <c r="I127" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J127" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7034,12 +7161,12 @@
       </c>
       <c r="I128" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J128" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7084,12 +7211,12 @@
       </c>
       <c r="I129" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J129" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7134,12 +7261,12 @@
       </c>
       <c r="I130" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J130" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7184,12 +7311,12 @@
       </c>
       <c r="I131" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J131" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7234,12 +7361,12 @@
       </c>
       <c r="I132" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J132" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7284,12 +7411,12 @@
       </c>
       <c r="I133" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J133" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7334,12 +7461,12 @@
       </c>
       <c r="I134" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J134" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7384,12 +7511,12 @@
       </c>
       <c r="I135" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J135" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7434,12 +7561,12 @@
       </c>
       <c r="I136" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J136" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7484,12 +7611,12 @@
       </c>
       <c r="I137" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J137" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7534,12 +7661,12 @@
       </c>
       <c r="I138" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J138" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7584,12 +7711,12 @@
       </c>
       <c r="I139" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J139" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7634,12 +7761,12 @@
       </c>
       <c r="I140" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J140" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7684,12 +7811,12 @@
       </c>
       <c r="I141" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J141" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7734,12 +7861,12 @@
       </c>
       <c r="I142" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J142" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7784,12 +7911,12 @@
       </c>
       <c r="I143" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J143" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7834,12 +7961,12 @@
       </c>
       <c r="I144" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J144" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7884,12 +8011,12 @@
       </c>
       <c r="I145" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J145" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -7934,12 +8061,12 @@
       </c>
       <c r="I146" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J146" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -8134,12 +8261,12 @@
       </c>
       <c r="I150" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J150" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -8184,12 +8311,12 @@
       </c>
       <c r="I151" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J151" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -8234,12 +8361,12 @@
       </c>
       <c r="I152" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J152" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -8284,12 +8411,12 @@
       </c>
       <c r="I153" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J153" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -8334,12 +8461,12 @@
       </c>
       <c r="I154" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J154" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -8384,12 +8511,12 @@
       </c>
       <c r="I155" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J155" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -8434,12 +8561,12 @@
       </c>
       <c r="I156" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J156" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -8484,12 +8611,12 @@
       </c>
       <c r="I157" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J157" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -8534,12 +8661,12 @@
       </c>
       <c r="I158" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J158" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -8585,7 +8712,7 @@
       </c>
       <c r="J159" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -8631,7 +8758,7 @@
       </c>
       <c r="J160" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -8677,7 +8804,7 @@
       </c>
       <c r="J161" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -8723,7 +8850,7 @@
       </c>
       <c r="J162" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -8769,7 +8896,7 @@
       </c>
       <c r="J163" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -8815,7 +8942,7 @@
       </c>
       <c r="J164" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -8861,7 +8988,7 @@
       </c>
       <c r="J165" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -8907,7 +9034,7 @@
       </c>
       <c r="J166" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -8952,12 +9079,12 @@
       </c>
       <c r="I167" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J167" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9002,12 +9129,12 @@
       </c>
       <c r="I168" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J168" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9052,12 +9179,12 @@
       </c>
       <c r="I169" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J169" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9102,12 +9229,12 @@
       </c>
       <c r="I170" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J170" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9152,12 +9279,12 @@
       </c>
       <c r="I171" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J171" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9352,12 +9479,12 @@
       </c>
       <c r="I175" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J175" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9402,12 +9529,12 @@
       </c>
       <c r="I176" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J176" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9452,12 +9579,12 @@
       </c>
       <c r="I177" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J177" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9502,12 +9629,12 @@
       </c>
       <c r="I178" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J178" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9552,12 +9679,12 @@
       </c>
       <c r="I179" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J179" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9602,12 +9729,12 @@
       </c>
       <c r="I180" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J180" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9652,12 +9779,12 @@
       </c>
       <c r="I181" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J181" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9702,12 +9829,12 @@
       </c>
       <c r="I182" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J182" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9752,12 +9879,12 @@
       </c>
       <c r="I183" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J183" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9802,12 +9929,12 @@
       </c>
       <c r="I184" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J184" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9852,12 +9979,12 @@
       </c>
       <c r="I185" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J185" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9902,12 +10029,12 @@
       </c>
       <c r="I186" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J186" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -9952,12 +10079,12 @@
       </c>
       <c r="I187" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J187" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -10002,12 +10129,12 @@
       </c>
       <c r="I188" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J188" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -10052,12 +10179,12 @@
       </c>
       <c r="I189" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J189" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -10102,12 +10229,12 @@
       </c>
       <c r="I190" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J190" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -10202,12 +10329,12 @@
       </c>
       <c r="I192" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J192" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -10252,12 +10379,12 @@
       </c>
       <c r="I193" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J193" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -10302,12 +10429,12 @@
       </c>
       <c r="I194" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J194" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -10352,12 +10479,12 @@
       </c>
       <c r="I195" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J195" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -10402,12 +10529,12 @@
       </c>
       <c r="I196" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J196" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -10552,12 +10679,12 @@
       </c>
       <c r="I199" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J199" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -10853,7 +10980,7 @@
       </c>
       <c r="J205" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -11248,12 +11375,12 @@
       </c>
       <c r="I213" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J213" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -11348,12 +11475,12 @@
       </c>
       <c r="I215" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J215" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -11548,12 +11675,12 @@
       </c>
       <c r="I219" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J219" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -11749,7 +11876,7 @@
       </c>
       <c r="J223" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -11794,12 +11921,12 @@
       </c>
       <c r="I224" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J224" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -11894,12 +12021,12 @@
       </c>
       <c r="I226" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J226" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -12044,12 +12171,12 @@
       </c>
       <c r="I229" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J229" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -12144,12 +12271,12 @@
       </c>
       <c r="I231" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J231" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -12194,12 +12321,12 @@
       </c>
       <c r="I232" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J232" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -12294,12 +12421,12 @@
       </c>
       <c r="I234" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J234" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -12494,12 +12621,12 @@
       </c>
       <c r="I238" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J238" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -12645,7 +12772,7 @@
       </c>
       <c r="J241" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -13190,12 +13317,12 @@
       </c>
       <c r="I252" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J252" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -13290,12 +13417,12 @@
       </c>
       <c r="I254" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J254" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -13490,12 +13617,12 @@
       </c>
       <c r="I258" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J258" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -13541,7 +13668,7 @@
       </c>
       <c r="J259" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -13636,12 +13763,12 @@
       </c>
       <c r="I261" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J261" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -13736,12 +13863,12 @@
       </c>
       <c r="I263" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J263" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -13886,12 +14013,12 @@
       </c>
       <c r="I266" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J266" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -14136,12 +14263,12 @@
       </c>
       <c r="I271" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J271" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -14236,12 +14363,12 @@
       </c>
       <c r="I273" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J273" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dipakai untuk memahami cara pengguna mencari; tidak ditulis sebagai klaim promo, termurah, terbaik, atau viral.</t>
         </is>
       </c>
     </row>
@@ -14437,7 +14564,7 @@
       </c>
       <c r="J277" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -15833,7 +15960,7 @@
       </c>
       <c r="J305" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -16729,7 +16856,7 @@
       </c>
       <c r="J323" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -17625,7 +17752,7 @@
       </c>
       <c r="J341" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -18521,7 +18648,7 @@
       </c>
       <c r="J359" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -19417,7 +19544,7 @@
       </c>
       <c r="J377" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -20102,12 +20229,12 @@
       </c>
       <c r="G391" s="11" t="inlineStr">
         <is>
-          <t>/tentang</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H391" s="11" t="inlineStr">
         <is>
-          <t>Entity &amp; trust</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I391" s="11" t="inlineStr">
@@ -20117,7 +20244,7 @@
       </c>
       <c r="J391" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20152,12 +20279,12 @@
       </c>
       <c r="G392" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H392" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I392" s="11" t="inlineStr">
@@ -20167,7 +20294,7 @@
       </c>
       <c r="J392" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20202,12 +20329,12 @@
       </c>
       <c r="G393" s="11" t="inlineStr">
         <is>
-          <t>/dimsum-cake</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H393" s="11" t="inlineStr">
         <is>
-          <t>Cake &amp; celebration</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I393" s="11" t="inlineStr">
@@ -20217,7 +20344,7 @@
       </c>
       <c r="J393" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20252,12 +20379,12 @@
       </c>
       <c r="G394" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H394" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I394" s="11" t="inlineStr">
@@ -20267,7 +20394,7 @@
       </c>
       <c r="J394" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20302,12 +20429,12 @@
       </c>
       <c r="G395" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H395" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I395" s="11" t="inlineStr">
@@ -20317,7 +20444,7 @@
       </c>
       <c r="J395" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20352,12 +20479,12 @@
       </c>
       <c r="G396" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H396" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I396" s="11" t="inlineStr">
@@ -20367,7 +20494,7 @@
       </c>
       <c r="J396" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20403,17 +20530,17 @@
       <c r="G397" s="11" t="inlineStr"/>
       <c r="H397" s="11" t="inlineStr">
         <is>
-          <t>Backlog artikel</t>
+          <t>Butuh SOP client</t>
         </is>
       </c>
       <c r="I397" s="11" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Butuh verifikasi</t>
         </is>
       </c>
       <c r="J397" s="12" t="inlineStr">
         <is>
-          <t>Kandidat artikel first-party; bukan alasan membuat halaman tipis.</t>
+          <t>Belum dipublikasikan agar tidak mengarang panduan penyimpanan atau pemanasan produk.</t>
         </is>
       </c>
     </row>
@@ -20449,17 +20576,17 @@
       <c r="G398" s="11" t="inlineStr"/>
       <c r="H398" s="11" t="inlineStr">
         <is>
-          <t>Backlog artikel</t>
+          <t>Butuh SOP client</t>
         </is>
       </c>
       <c r="I398" s="11" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Butuh verifikasi</t>
         </is>
       </c>
       <c r="J398" s="12" t="inlineStr">
         <is>
-          <t>Kandidat artikel first-party; bukan alasan membuat halaman tipis.</t>
+          <t>Belum dipublikasikan agar tidak mengarang panduan penyimpanan atau pemanasan produk.</t>
         </is>
       </c>
     </row>
@@ -20494,12 +20621,12 @@
       </c>
       <c r="G399" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H399" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I399" s="11" t="inlineStr">
@@ -20509,7 +20636,7 @@
       </c>
       <c r="J399" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20545,17 +20672,17 @@
       <c r="G400" s="11" t="inlineStr"/>
       <c r="H400" s="11" t="inlineStr">
         <is>
-          <t>Backlog artikel</t>
+          <t>Butuh SOP client</t>
         </is>
       </c>
       <c r="I400" s="11" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Butuh verifikasi</t>
         </is>
       </c>
       <c r="J400" s="12" t="inlineStr">
         <is>
-          <t>Kandidat artikel first-party; bukan alasan membuat halaman tipis.</t>
+          <t>Belum dipublikasikan agar tidak mengarang panduan penyimpanan atau pemanasan produk.</t>
         </is>
       </c>
     </row>
@@ -20591,17 +20718,17 @@
       <c r="G401" s="11" t="inlineStr"/>
       <c r="H401" s="11" t="inlineStr">
         <is>
-          <t>Backlog artikel</t>
+          <t>Butuh SOP client</t>
         </is>
       </c>
       <c r="I401" s="11" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Butuh verifikasi</t>
         </is>
       </c>
       <c r="J401" s="12" t="inlineStr">
         <is>
-          <t>Kandidat artikel first-party; bukan alasan membuat halaman tipis.</t>
+          <t>Belum dipublikasikan agar tidak mengarang panduan penyimpanan atau pemanasan produk.</t>
         </is>
       </c>
     </row>
@@ -20636,12 +20763,12 @@
       </c>
       <c r="G402" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H402" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I402" s="11" t="inlineStr">
@@ -20651,7 +20778,7 @@
       </c>
       <c r="J402" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20686,12 +20813,12 @@
       </c>
       <c r="G403" s="11" t="inlineStr">
         <is>
-          <t>/dimsum-cake</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H403" s="11" t="inlineStr">
         <is>
-          <t>Cake &amp; celebration</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I403" s="11" t="inlineStr">
@@ -20701,7 +20828,7 @@
       </c>
       <c r="J403" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20736,12 +20863,12 @@
       </c>
       <c r="G404" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H404" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I404" s="11" t="inlineStr">
@@ -20751,7 +20878,7 @@
       </c>
       <c r="J404" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20786,12 +20913,12 @@
       </c>
       <c r="G405" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H405" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I405" s="11" t="inlineStr">
@@ -20801,7 +20928,7 @@
       </c>
       <c r="J405" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20836,12 +20963,12 @@
       </c>
       <c r="G406" s="11" t="inlineStr">
         <is>
-          <t>/dimsum-cake</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H406" s="11" t="inlineStr">
         <is>
-          <t>Cake &amp; celebration</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I406" s="11" t="inlineStr">
@@ -20851,7 +20978,7 @@
       </c>
       <c r="J406" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20886,12 +21013,12 @@
       </c>
       <c r="G407" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H407" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I407" s="11" t="inlineStr">
@@ -20901,7 +21028,7 @@
       </c>
       <c r="J407" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20936,12 +21063,12 @@
       </c>
       <c r="G408" s="11" t="inlineStr">
         <is>
-          <t>/dimsum-cake</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H408" s="11" t="inlineStr">
         <is>
-          <t>Cake &amp; celebration</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I408" s="11" t="inlineStr">
@@ -20951,7 +21078,7 @@
       </c>
       <c r="J408" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -20986,12 +21113,12 @@
       </c>
       <c r="G409" s="11" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H409" s="11" t="inlineStr">
         <is>
-          <t>Local intent</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I409" s="11" t="inlineStr">
@@ -21001,7 +21128,7 @@
       </c>
       <c r="J409" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21036,12 +21163,12 @@
       </c>
       <c r="G410" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H410" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I410" s="11" t="inlineStr">
@@ -21051,7 +21178,7 @@
       </c>
       <c r="J410" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21084,20 +21211,24 @@
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="G411" s="11" t="inlineStr"/>
+      <c r="G411" s="11" t="inlineStr">
+        <is>
+          <t>/faq</t>
+        </is>
+      </c>
       <c r="H411" s="11" t="inlineStr">
         <is>
-          <t>Backlog artikel</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I411" s="11" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Diimplementasikan</t>
         </is>
       </c>
       <c r="J411" s="12" t="inlineStr">
         <is>
-          <t>Kandidat artikel first-party; bukan alasan membuat halaman tipis.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21132,12 +21263,12 @@
       </c>
       <c r="G412" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H412" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I412" s="11" t="inlineStr">
@@ -21147,7 +21278,7 @@
       </c>
       <c r="J412" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21182,12 +21313,12 @@
       </c>
       <c r="G413" s="11" t="inlineStr">
         <is>
-          <t>/dimsum-cake</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H413" s="11" t="inlineStr">
         <is>
-          <t>Cake &amp; celebration</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I413" s="11" t="inlineStr">
@@ -21197,7 +21328,7 @@
       </c>
       <c r="J413" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21232,12 +21363,12 @@
       </c>
       <c r="G414" s="11" t="inlineStr">
         <is>
-          <t>/tentang</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H414" s="11" t="inlineStr">
         <is>
-          <t>Entity &amp; trust</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I414" s="11" t="inlineStr">
@@ -21247,7 +21378,7 @@
       </c>
       <c r="J414" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21282,12 +21413,12 @@
       </c>
       <c r="G415" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H415" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I415" s="11" t="inlineStr">
@@ -21297,7 +21428,7 @@
       </c>
       <c r="J415" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21332,12 +21463,12 @@
       </c>
       <c r="G416" s="11" t="inlineStr">
         <is>
-          <t>/tentang</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H416" s="11" t="inlineStr">
         <is>
-          <t>Entity &amp; trust</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I416" s="11" t="inlineStr">
@@ -21347,7 +21478,7 @@
       </c>
       <c r="J416" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21382,12 +21513,12 @@
       </c>
       <c r="G417" s="11" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H417" s="11" t="inlineStr">
         <is>
-          <t>Local intent</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I417" s="11" t="inlineStr">
@@ -21397,7 +21528,7 @@
       </c>
       <c r="J417" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21432,12 +21563,12 @@
       </c>
       <c r="G418" s="11" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H418" s="11" t="inlineStr">
         <is>
-          <t>Local intent</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I418" s="11" t="inlineStr">
@@ -21447,7 +21578,7 @@
       </c>
       <c r="J418" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21482,12 +21613,12 @@
       </c>
       <c r="G419" s="11" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H419" s="11" t="inlineStr">
         <is>
-          <t>Local intent</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I419" s="11" t="inlineStr">
@@ -21497,7 +21628,7 @@
       </c>
       <c r="J419" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21532,12 +21663,12 @@
       </c>
       <c r="G420" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H420" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I420" s="11" t="inlineStr">
@@ -21547,7 +21678,7 @@
       </c>
       <c r="J420" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21582,12 +21713,12 @@
       </c>
       <c r="G421" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H421" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I421" s="11" t="inlineStr">
@@ -21597,7 +21728,7 @@
       </c>
       <c r="J421" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21632,12 +21763,12 @@
       </c>
       <c r="G422" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H422" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I422" s="11" t="inlineStr">
@@ -21647,7 +21778,7 @@
       </c>
       <c r="J422" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21682,12 +21813,12 @@
       </c>
       <c r="G423" s="11" t="inlineStr">
         <is>
-          <t>/dimsum-cake</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H423" s="11" t="inlineStr">
         <is>
-          <t>Cake &amp; celebration</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I423" s="11" t="inlineStr">
@@ -21697,7 +21828,7 @@
       </c>
       <c r="J423" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21732,12 +21863,12 @@
       </c>
       <c r="G424" s="11" t="inlineStr">
         <is>
-          <t>/tentang</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H424" s="11" t="inlineStr">
         <is>
-          <t>Entity &amp; trust</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I424" s="11" t="inlineStr">
@@ -21747,7 +21878,7 @@
       </c>
       <c r="J424" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21782,12 +21913,12 @@
       </c>
       <c r="G425" s="11" t="inlineStr">
         <is>
-          <t>/dimsum-cake</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H425" s="11" t="inlineStr">
         <is>
-          <t>Cake &amp; celebration</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I425" s="11" t="inlineStr">
@@ -21797,7 +21928,7 @@
       </c>
       <c r="J425" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21832,12 +21963,12 @@
       </c>
       <c r="G426" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H426" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I426" s="11" t="inlineStr">
@@ -21847,7 +21978,7 @@
       </c>
       <c r="J426" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21882,12 +22013,12 @@
       </c>
       <c r="G427" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H427" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I427" s="11" t="inlineStr">
@@ -21897,7 +22028,7 @@
       </c>
       <c r="J427" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21932,12 +22063,12 @@
       </c>
       <c r="G428" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H428" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I428" s="11" t="inlineStr">
@@ -21947,7 +22078,7 @@
       </c>
       <c r="J428" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -21982,12 +22113,12 @@
       </c>
       <c r="G429" s="11" t="inlineStr">
         <is>
-          <t>/dimsum-cake</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H429" s="11" t="inlineStr">
         <is>
-          <t>Cake &amp; celebration</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I429" s="11" t="inlineStr">
@@ -21997,7 +22128,7 @@
       </c>
       <c r="J429" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22032,12 +22163,12 @@
       </c>
       <c r="G430" s="11" t="inlineStr">
         <is>
-          <t>/dimsum-cake</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H430" s="11" t="inlineStr">
         <is>
-          <t>Cake &amp; celebration</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I430" s="11" t="inlineStr">
@@ -22047,7 +22178,7 @@
       </c>
       <c r="J430" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22082,12 +22213,12 @@
       </c>
       <c r="G431" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H431" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I431" s="11" t="inlineStr">
@@ -22097,7 +22228,7 @@
       </c>
       <c r="J431" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22132,12 +22263,12 @@
       </c>
       <c r="G432" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H432" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I432" s="11" t="inlineStr">
@@ -22147,7 +22278,7 @@
       </c>
       <c r="J432" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22182,12 +22313,12 @@
       </c>
       <c r="G433" s="11" t="inlineStr">
         <is>
-          <t>/dimsum-cake</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H433" s="11" t="inlineStr">
         <is>
-          <t>Cake &amp; celebration</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I433" s="11" t="inlineStr">
@@ -22197,7 +22328,7 @@
       </c>
       <c r="J433" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan secara semantik melalui copy, tabel harga, FAQ, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22232,12 +22363,12 @@
       </c>
       <c r="G434" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H434" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I434" s="11" t="inlineStr">
@@ -22247,7 +22378,7 @@
       </c>
       <c r="J434" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22282,12 +22413,12 @@
       </c>
       <c r="G435" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H435" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I435" s="11" t="inlineStr">
@@ -22297,7 +22428,7 @@
       </c>
       <c r="J435" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22332,12 +22463,12 @@
       </c>
       <c r="G436" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H436" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I436" s="11" t="inlineStr">
@@ -22347,7 +22478,7 @@
       </c>
       <c r="J436" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22382,12 +22513,12 @@
       </c>
       <c r="G437" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H437" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I437" s="11" t="inlineStr">
@@ -22397,7 +22528,7 @@
       </c>
       <c r="J437" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22443,7 +22574,7 @@
       </c>
       <c r="J438" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -22489,7 +22620,7 @@
       </c>
       <c r="J439" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -22535,7 +22666,7 @@
       </c>
       <c r="J440" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -22570,12 +22701,12 @@
       </c>
       <c r="G441" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H441" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I441" s="11" t="inlineStr">
@@ -22585,7 +22716,7 @@
       </c>
       <c r="J441" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22620,12 +22751,12 @@
       </c>
       <c r="G442" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H442" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I442" s="11" t="inlineStr">
@@ -22635,7 +22766,7 @@
       </c>
       <c r="J442" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22670,12 +22801,12 @@
       </c>
       <c r="G443" s="11" t="inlineStr">
         <is>
-          <t>/pesanan-acara</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H443" s="11" t="inlineStr">
         <is>
-          <t>Acara &amp; bulk order</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I443" s="11" t="inlineStr">
@@ -22685,7 +22816,7 @@
       </c>
       <c r="J443" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22731,7 +22862,7 @@
       </c>
       <c r="J444" s="12" t="inlineStr">
         <is>
-          <t>Belum diterbitkan karena produk, kanal, atau layanan belum terverifikasi.</t>
+          <t>Tidak ditargetkan sampai client mengonfirmasi produk, kanal, atau layanan tersebut.</t>
         </is>
       </c>
     </row>
@@ -22766,12 +22897,12 @@
       </c>
       <c r="G445" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H445" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I445" s="11" t="inlineStr">
@@ -22781,7 +22912,7 @@
       </c>
       <c r="J445" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22816,12 +22947,12 @@
       </c>
       <c r="G446" s="11" t="inlineStr">
         <is>
-          <t>/tentang</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H446" s="11" t="inlineStr">
         <is>
-          <t>Entity &amp; trust</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I446" s="11" t="inlineStr">
@@ -22831,7 +22962,7 @@
       </c>
       <c r="J446" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22866,12 +22997,12 @@
       </c>
       <c r="G447" s="11" t="inlineStr">
         <is>
-          <t>/tentang</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H447" s="11" t="inlineStr">
         <is>
-          <t>Entity &amp; trust</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I447" s="11" t="inlineStr">
@@ -22881,7 +23012,7 @@
       </c>
       <c r="J447" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui fakta brand, lokasi, halal, jam layanan, dan kanal resmi.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22916,12 +23047,12 @@
       </c>
       <c r="G448" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H448" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I448" s="11" t="inlineStr">
@@ -22931,7 +23062,7 @@
       </c>
       <c r="J448" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -22966,12 +23097,12 @@
       </c>
       <c r="G449" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H449" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I449" s="11" t="inlineStr">
@@ -22981,7 +23112,7 @@
       </c>
       <c r="J449" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -23016,12 +23147,12 @@
       </c>
       <c r="G450" s="11" t="inlineStr">
         <is>
-          <t>/menu</t>
+          <t>/faq</t>
         </is>
       </c>
       <c r="H450" s="11" t="inlineStr">
         <is>
-          <t>Menu &amp; product</t>
+          <t>AEO / direct answers</t>
         </is>
       </c>
       <c r="I450" s="11" t="inlineStr">
@@ -23031,7 +23162,7 @@
       </c>
       <c r="J450" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dijawab pada FAQ resmi atau halaman intent terkait menggunakan fakta produk aktual.</t>
         </is>
       </c>
     </row>
@@ -23526,12 +23657,12 @@
       </c>
       <c r="I460" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J460" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -23576,12 +23707,12 @@
       </c>
       <c r="I461" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J461" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -23626,12 +23757,12 @@
       </c>
       <c r="I462" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J462" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -23676,12 +23807,12 @@
       </c>
       <c r="I463" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J463" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -23726,12 +23857,12 @@
       </c>
       <c r="I464" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J464" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -23776,12 +23907,12 @@
       </c>
       <c r="I465" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J465" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -23826,12 +23957,12 @@
       </c>
       <c r="I466" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J466" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -23876,12 +24007,12 @@
       </c>
       <c r="I467" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J467" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -23926,12 +24057,12 @@
       </c>
       <c r="I468" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J468" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -23976,12 +24107,12 @@
       </c>
       <c r="I469" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J469" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24026,12 +24157,12 @@
       </c>
       <c r="I470" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J470" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24076,12 +24207,12 @@
       </c>
       <c r="I471" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J471" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24126,12 +24257,12 @@
       </c>
       <c r="I472" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J472" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24176,12 +24307,12 @@
       </c>
       <c r="I473" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J473" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24226,12 +24357,12 @@
       </c>
       <c r="I474" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J474" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24276,12 +24407,12 @@
       </c>
       <c r="I475" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J475" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24326,12 +24457,12 @@
       </c>
       <c r="I476" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J476" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24376,12 +24507,12 @@
       </c>
       <c r="I477" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J477" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24426,12 +24557,12 @@
       </c>
       <c r="I478" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J478" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24476,12 +24607,12 @@
       </c>
       <c r="I479" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J479" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24526,12 +24657,12 @@
       </c>
       <c r="I480" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J480" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24576,12 +24707,12 @@
       </c>
       <c r="I481" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J481" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24626,12 +24757,12 @@
       </c>
       <c r="I482" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J482" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24676,12 +24807,12 @@
       </c>
       <c r="I483" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J483" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24726,12 +24857,12 @@
       </c>
       <c r="I484" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J484" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24776,12 +24907,12 @@
       </c>
       <c r="I485" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J485" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24826,12 +24957,12 @@
       </c>
       <c r="I486" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J486" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24876,12 +25007,12 @@
       </c>
       <c r="I487" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J487" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24926,12 +25057,12 @@
       </c>
       <c r="I488" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J488" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -24976,12 +25107,12 @@
       </c>
       <c r="I489" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J489" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -25026,12 +25157,12 @@
       </c>
       <c r="I490" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J490" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -25076,12 +25207,12 @@
       </c>
       <c r="I491" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J491" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -25126,12 +25257,12 @@
       </c>
       <c r="I492" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J492" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -25176,12 +25307,12 @@
       </c>
       <c r="I493" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J493" s="12" t="inlineStr">
         <is>
-          <t>Dikonsolidasikan ke homepage/local entity tanpa membuat doorway page per wilayah.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -25226,12 +25357,12 @@
       </c>
       <c r="I494" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J494" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui informasi ukuran, harga, kebutuhan acara, dan SOP pengiriman.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -25276,12 +25407,12 @@
       </c>
       <c r="I495" s="11" t="inlineStr">
         <is>
-          <t>Diimplementasikan</t>
+          <t>Variasi semantik</t>
         </is>
       </c>
       <c r="J495" s="12" t="inlineStr">
         <is>
-          <t>Ditargetkan melalui katalog aktual, harga, direct answers, dan Product/Offer.</t>
+          <t>Dicakup melalui area layanan Jabodetabek; tidak dibuat sebagai doorway page untuk setiap wilayah.</t>
         </is>
       </c>
     </row>
@@ -25591,7 +25722,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>